<commit_message>
Added sprint2 docs and added doc folders
</commit_message>
<xml_diff>
--- a/docs/project_backlog.xlsx
+++ b/docs/project_backlog.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>ID</t>
   </si>
@@ -22,7 +22,7 @@
     <t>Estimation (hours)</t>
   </si>
   <si>
-    <t>Priority (1-5)</t>
+    <t>Priority (1-3)</t>
   </si>
   <si>
     <t>Sprint When Finished</t>
@@ -61,25 +61,115 @@
     <t>Add event markers and response indicators to visualizations</t>
   </si>
   <si>
+    <t>Fix epoch times to autocorrect if out of bounds</t>
+  </si>
+  <si>
+    <t>Tabbed view for multiple files</t>
+  </si>
+  <si>
+    <t>Save graph button</t>
+  </si>
+  <si>
+    <t>Package application as standalone executable with PyInstaller</t>
+  </si>
+  <si>
+    <t>UI updates</t>
+  </si>
+  <si>
+    <t>Fix topo map for fewer sensors</t>
+  </si>
+  <si>
+    <t>Research ganglion data repo</t>
+  </si>
+  <si>
+    <t>Parsing .set file better for cyber security and check magic numbers on csv files</t>
+  </si>
+  <si>
+    <t>Change live mode button to open flanker task/eeg generator</t>
+  </si>
+  <si>
+    <t>Select multiple channels (checkbox)</t>
+  </si>
+  <si>
+    <t>Adding flag that allows to pass into file path to auto load instead of browse (for testing purposes)</t>
+  </si>
+  <si>
+    <t>Convert csv to .set</t>
+  </si>
+  <si>
+    <t>Pressing 'enter' now lets user reload</t>
+  </si>
+  <si>
+    <t>Create a log system so unless we run it with the system in a debug mode we do not output info to terminal</t>
+  </si>
+  <si>
+    <t>Get app running in cloud</t>
+  </si>
+  <si>
+    <t>Icon for application</t>
+  </si>
+  <si>
+    <t>Event dropdown (highlight/show different event epochs/time occured ?)</t>
+  </si>
+  <si>
+    <t>Updating help dialog to either be our ReadMe or update ReadMe to reflect the help dialog</t>
+  </si>
+  <si>
     <t>Detect ErrPs in real-time during task execution</t>
   </si>
   <si>
     <t xml:space="preserve">Integrate with PsyToolkit flanker task </t>
   </si>
   <si>
-    <t>Implement real-time EEG signal processing and classification</t>
-  </si>
-  <si>
     <t>Handle continuous (non-epoched) EEG data</t>
   </si>
   <si>
-    <t>Create block-based visual interface similar to scratch</t>
-  </si>
-  <si>
     <t>Implement tools for ErrP detection</t>
   </si>
   <si>
-    <t>Package application as standalone executable with PyInstaller</t>
+    <t>Documentation per function (input, output, functionality)</t>
+  </si>
+  <si>
+    <t>Update ReadMe</t>
+  </si>
+  <si>
+    <t>Update help button to parse readme on github so if readme is updated the help is updated</t>
+  </si>
+  <si>
+    <t>Code cleanup</t>
+  </si>
+  <si>
+    <t>Test with OpenBCI Ganglion</t>
+  </si>
+  <si>
+    <t>Project site update with documentation</t>
+  </si>
+  <si>
+    <t>Unit tests</t>
+  </si>
+  <si>
+    <t>Add final executable to repo</t>
+  </si>
+  <si>
+    <t>Icon once pyinstaller is working</t>
+  </si>
+  <si>
+    <t>Add flag info to ReadMe</t>
+  </si>
+  <si>
+    <t>User guide doc</t>
+  </si>
+  <si>
+    <t>Development guide doc (how to modify)</t>
+  </si>
+  <si>
+    <t>Install/Deployment guide doc</t>
+  </si>
+  <si>
+    <t>Test plan/cases doc</t>
+  </si>
+  <si>
+    <t>FAQs/Gotchas doc</t>
   </si>
 </sst>
 </file>
@@ -99,12 +189,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor rgb="FFF6F8F9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -113,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -129,9 +225,23 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -336,12 +446,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E19" displayName="Table1" name="Table1" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E49" displayName="Table1" name="Table1" id="1">
   <tableColumns count="5">
     <tableColumn name="ID" id="1"/>
     <tableColumn name="Story" id="2"/>
     <tableColumn name="Estimation (hours)" id="3"/>
-    <tableColumn name="Priority (1-5)" id="4"/>
+    <tableColumn name="Priority (1-3)" id="4"/>
     <tableColumn name="Sprint When Finished" id="5"/>
   </tableColumns>
   <tableStyleInfo name="Sheet1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
@@ -551,11 +661,12 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="4.13"/>
-    <col customWidth="1" min="2" max="2" width="67.13"/>
+    <col customWidth="1" min="2" max="2" width="80.13"/>
     <col customWidth="1" min="3" max="3" width="22.5"/>
     <col customWidth="1" min="4" max="4" width="14.63"/>
-    <col customWidth="1" min="5" max="5" width="26.25"/>
-    <col customWidth="1" min="6" max="26" width="14.38"/>
+    <col customWidth="1" min="5" max="5" width="20.5"/>
+    <col customWidth="1" min="6" max="6" width="17.75"/>
+    <col customWidth="1" min="7" max="26" width="14.38"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -659,7 +770,6 @@
       <c r="E6" s="4">
         <v>1.0</v>
       </c>
-      <c r="F6" s="5"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="3">
@@ -771,10 +881,13 @@
         <v>16</v>
       </c>
       <c r="C13" s="3">
-        <v>8.0</v>
+        <v>2.0</v>
       </c>
       <c r="D13" s="4">
-        <v>1.0</v>
+        <v>2.0</v>
+      </c>
+      <c r="E13" s="4">
+        <v>2.0</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
@@ -785,10 +898,13 @@
         <v>17</v>
       </c>
       <c r="C14" s="3">
-        <v>10.0</v>
+        <v>2.0</v>
       </c>
       <c r="D14" s="4">
         <v>1.0</v>
+      </c>
+      <c r="E14" s="4">
+        <v>2.0</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
@@ -799,10 +915,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="3">
-        <v>10.0</v>
+        <v>2.0</v>
       </c>
       <c r="D15" s="4">
-        <v>1.0</v>
+        <v>3.0</v>
+      </c>
+      <c r="E15" s="4">
+        <v>2.0</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
@@ -813,12 +932,14 @@
         <v>19</v>
       </c>
       <c r="C16" s="3">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="D16" s="4">
         <v>1.0</v>
       </c>
-      <c r="F16" s="5"/>
+      <c r="E16" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="3">
@@ -828,12 +949,14 @@
         <v>20</v>
       </c>
       <c r="C17" s="3">
-        <v>12.0</v>
+        <v>6.0</v>
       </c>
       <c r="D17" s="4">
         <v>2.0</v>
       </c>
-      <c r="F17" s="5"/>
+      <c r="E17" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="3">
@@ -843,12 +966,14 @@
         <v>21</v>
       </c>
       <c r="C18" s="3">
-        <v>10.0</v>
+        <v>2.0</v>
       </c>
       <c r="D18" s="4">
         <v>1.0</v>
       </c>
-      <c r="F18" s="5"/>
+      <c r="E18" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="3">
@@ -858,88 +983,406 @@
         <v>22</v>
       </c>
       <c r="C19" s="3">
-        <v>6.0</v>
+        <v>2.0</v>
       </c>
       <c r="D19" s="4">
         <v>1.0</v>
       </c>
-      <c r="F19" s="5"/>
+      <c r="E19" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="6"/>
-      <c r="B20" s="5"/>
-      <c r="F20" s="5"/>
+      <c r="A20" s="3">
+        <v>19.0</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="E20" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="6"/>
+      <c r="A21" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D21" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="E21" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="6"/>
-      <c r="B22" s="5"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
+      <c r="A22" s="3">
+        <v>21.0</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D22" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="E22" s="4">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="3">
+        <v>22.0</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D23" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="E23" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="5"/>
+      <c r="A24" s="3">
+        <v>23.0</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D24" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="E24" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="F25" s="5"/>
+      <c r="A25" s="3">
+        <v>24.0</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="D25" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="E25" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="B26" s="5"/>
-      <c r="F26" s="5"/>
+      <c r="A26" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2.0</v>
+      </c>
+      <c r="E26" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="5"/>
-      <c r="B27" s="5"/>
-      <c r="F27" s="5"/>
+      <c r="A27" s="3">
+        <v>26.0</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="D27" s="4">
+        <v>1.0</v>
+      </c>
+      <c r="E27" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="5"/>
-      <c r="B28" s="5"/>
+      <c r="A28" s="3">
+        <v>27.0</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="D28" s="4">
+        <v>3.0</v>
+      </c>
+      <c r="E28" s="4"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="5"/>
-      <c r="B29" s="5"/>
+      <c r="A29" s="3">
+        <v>28.0</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="D29" s="4">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
+      <c r="A30" s="3">
+        <v>29.0</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="D30" s="4">
+        <v>2.0</v>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="5"/>
-      <c r="B31" s="5"/>
+      <c r="A31" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C31" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="D31" s="4">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="5"/>
-      <c r="B32" s="5"/>
+      <c r="A32" s="3">
+        <v>31.0</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="D32" s="4">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="5"/>
-      <c r="B33" s="5"/>
+      <c r="A33" s="3">
+        <v>32.0</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C33" s="3">
+        <v>12.0</v>
+      </c>
+      <c r="D33" s="4">
+        <v>1.0</v>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="5"/>
-    </row>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
-    <row r="40" ht="15.75" customHeight="1"/>
-    <row r="41" ht="15.75" customHeight="1"/>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
-    <row r="49" ht="15.75" customHeight="1"/>
+      <c r="A34" s="3">
+        <v>33.0</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C34" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="D34" s="4">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="3">
+        <v>34.0</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="7"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="8"/>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="3">
+        <v>35.0</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="7"/>
+      <c r="D36" s="6"/>
+      <c r="E36" s="8"/>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="3">
+        <v>36.0</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C37" s="7"/>
+      <c r="D37" s="6"/>
+      <c r="E37" s="8"/>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="3">
+        <v>37.0</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" s="9"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="3">
+        <v>38.0</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" s="9"/>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="3">
+        <v>39.0</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C40" s="9"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="3">
+        <v>40.0</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C41" s="9"/>
+      <c r="D41" s="4">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="3">
+        <v>41.0</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C42" s="9"/>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="3">
+        <v>42.0</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C43" s="9"/>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="3">
+        <v>43.0</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="10"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="3">
+        <v>44.0</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="10"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="3">
+        <v>45.0</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="10"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="3">
+        <v>46.0</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C47" s="10"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" s="3">
+        <v>47.0</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C48" s="10"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="A49" s="3">
+        <v>48.0</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C49" s="10"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+    </row>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -1884,79 +2327,71 @@
     <row r="991" ht="15.75" customHeight="1"/>
     <row r="992" ht="15.75" customHeight="1"/>
     <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
-    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
-  <conditionalFormatting sqref="C2:C30">
+  <conditionalFormatting sqref="C2:C103">
     <cfRule type="cellIs" dxfId="5" priority="1" operator="lessThanOrEqual">
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C30">
+  <conditionalFormatting sqref="C2:C103">
     <cfRule type="cellIs" dxfId="6" priority="2" operator="between">
       <formula>4</formula>
       <formula>6</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C30">
+  <conditionalFormatting sqref="C2:C103">
     <cfRule type="cellIs" dxfId="7" priority="3" operator="between">
       <formula>7</formula>
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C30">
+  <conditionalFormatting sqref="C2:C103">
     <cfRule type="cellIs" dxfId="8" priority="4" operator="greaterThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D30">
+  <conditionalFormatting sqref="D2:D49">
     <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D30">
+  <conditionalFormatting sqref="D2:D49">
     <cfRule type="cellIs" dxfId="10" priority="6" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D30">
+  <conditionalFormatting sqref="D2:D49">
     <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E30">
+  <conditionalFormatting sqref="E2:E57">
     <cfRule type="cellIs" dxfId="12" priority="8" operator="equal">
       <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E30">
+  <conditionalFormatting sqref="E2:E57">
     <cfRule type="cellIs" dxfId="13" priority="9" operator="equal">
       <formula>2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E30">
+  <conditionalFormatting sqref="E2:E57">
     <cfRule type="cellIs" dxfId="14" priority="10" operator="equal">
       <formula>3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D30">
+  <conditionalFormatting sqref="D2:D49">
     <cfRule type="cellIs" dxfId="15" priority="11" operator="equal">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D16">
+  <conditionalFormatting sqref="D33">
     <cfRule type="cellIs" dxfId="16" priority="12" operator="equal">
       <formula>5</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A19 C2:C19">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A49 C2:C49">
       <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D")))))</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>